<commit_message>
cartes mono observatoires, graphs corrigés
</commit_message>
<xml_diff>
--- a/docs/downloads/04/tbl_cm_act_alaotra_tous.xlsx
+++ b/docs/downloads/04/tbl_cm_act_alaotra_tous.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -498,14 +498,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
+          <t>Inactif / Retraité</t>
         </is>
       </c>
       <c r="C9">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="D9">
-        <v>25.4</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="10">
@@ -516,32 +516,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Services &amp; Autres</t>
+          <t>Ouvrier agricole</t>
         </is>
       </c>
       <c r="C10">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="D10">
-        <v>13.4</v>
+        <v>25.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ambodivoara</t>
+          <t>Ambatomanga</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Artisanat, BTP &amp; Transport</t>
-        </is>
-      </c>
-      <c r="C11">
-        <v>6</v>
-      </c>
-      <c r="D11">
-        <v>10.3</v>
+          <t>Services &amp; Autres</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -552,8 +546,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Commerce &amp; Restauration</t>
-        </is>
+          <t>Artisanat, BTP &amp; Transport</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>6</v>
+      </c>
+      <c r="D12">
+        <v>10.3</v>
       </c>
     </row>
     <row r="13">
@@ -564,14 +564,8 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cultivateur exploitant</t>
-        </is>
-      </c>
-      <c r="C13">
-        <v>38</v>
-      </c>
-      <c r="D13">
-        <v>65.5</v>
+          <t>Commerce &amp; Restauration</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -582,8 +576,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Elevage, Pêche &amp; Ress. nat.</t>
-        </is>
+          <t>Cultivateur exploitant</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>38</v>
+      </c>
+      <c r="D14">
+        <v>65.5</v>
       </c>
     </row>
     <row r="15">
@@ -594,14 +594,8 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
-        </is>
-      </c>
-      <c r="C15">
-        <v>6</v>
-      </c>
-      <c r="D15">
-        <v>10.3</v>
+          <t>Elevage, Pêche &amp; Ress. nat.</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -612,26 +606,26 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Services &amp; Autres</t>
+          <t>Inactif / Retraité</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Ambohidrony</t>
+          <t>Ambodivoara</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Artisanat, BTP &amp; Transport</t>
+          <t>Ouvrier agricole</t>
         </is>
       </c>
       <c r="C17">
         <v>6</v>
       </c>
       <c r="D17">
-        <v>11.5</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="18">
@@ -642,8 +636,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Commerce &amp; Restauration</t>
-        </is>
+          <t>Artisanat, BTP &amp; Transport</t>
+        </is>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <v>11.5</v>
       </c>
     </row>
     <row r="19">
@@ -654,14 +654,8 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cultivateur exploitant</t>
-        </is>
-      </c>
-      <c r="C19">
-        <v>19</v>
-      </c>
-      <c r="D19">
-        <v>36.5</v>
+          <t>Commerce &amp; Restauration</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -672,14 +666,14 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Elevage, Pêche &amp; Ress. nat.</t>
+          <t>Cultivateur exploitant</t>
         </is>
       </c>
       <c r="C20">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="D20">
-        <v>11.5</v>
+        <v>36.5</v>
       </c>
     </row>
     <row r="21">
@@ -690,14 +684,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
+          <t>Elevage, Pêche &amp; Ress. nat.</t>
         </is>
       </c>
       <c r="C21">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D21">
-        <v>26.9</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="22">
@@ -708,38 +702,38 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Services &amp; Autres</t>
+          <t>Inactif / Retraité</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Analamiranga</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Artisanat, BTP &amp; Transport</t>
-        </is>
+          <t>Ouvrier agricole</t>
+        </is>
+      </c>
+      <c r="C23">
+        <v>14</v>
+      </c>
+      <c r="D23">
+        <v>26.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Analamiranga</t>
+          <t>Ambohidrony</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Commerce &amp; Restauration</t>
-        </is>
-      </c>
-      <c r="C24">
-        <v>5</v>
-      </c>
-      <c r="D24">
-        <v>10.9</v>
+          <t>Services &amp; Autres</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -750,14 +744,8 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cultivateur exploitant</t>
-        </is>
-      </c>
-      <c r="C25">
-        <v>28</v>
-      </c>
-      <c r="D25">
-        <v>60.9</v>
+          <t>Artisanat, BTP &amp; Transport</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -768,14 +756,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
+          <t>Commerce &amp; Restauration</t>
         </is>
       </c>
       <c r="C26">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D26">
-        <v>13</v>
+        <v>10.9</v>
       </c>
     </row>
     <row r="27">
@@ -786,56 +774,56 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Services &amp; Autres</t>
-        </is>
+          <t>Cultivateur exploitant</t>
+        </is>
+      </c>
+      <c r="C27">
+        <v>28</v>
+      </c>
+      <c r="D27">
+        <v>60.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Avaradrano</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Artisanat, BTP &amp; Transport</t>
-        </is>
-      </c>
-      <c r="C28">
-        <v>6</v>
-      </c>
-      <c r="D28">
-        <v>6.7</v>
+          <t>Inactif / Retraité</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Avaradrano</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Commerce &amp; Restauration</t>
-        </is>
+          <t>Ouvrier agricole</t>
+        </is>
+      </c>
+      <c r="C29">
+        <v>6</v>
+      </c>
+      <c r="D29">
+        <v>13</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Avaradrano</t>
+          <t>Analamiranga</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cultivateur exploitant</t>
-        </is>
-      </c>
-      <c r="C30">
-        <v>65</v>
-      </c>
-      <c r="D30">
-        <v>73</v>
+          <t>Services &amp; Autres</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -846,7 +834,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Elevage, Pêche &amp; Ress. nat.</t>
+          <t>Artisanat, BTP &amp; Transport</t>
         </is>
       </c>
       <c r="C31">
@@ -864,7 +852,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
+          <t>Commerce &amp; Restauration</t>
         </is>
       </c>
     </row>
@@ -876,79 +864,67 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Services &amp; Autres</t>
+          <t>Cultivateur exploitant</t>
         </is>
       </c>
       <c r="C33">
-        <v>7</v>
+        <v>65</v>
       </c>
       <c r="D33">
-        <v>7.9</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Feramanga Atsimo</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Artisanat, BTP &amp; Transport</t>
+          <t>Elevage, Pêche &amp; Ress. nat.</t>
         </is>
       </c>
       <c r="C34">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D34">
-        <v>5.6</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Feramanga Atsimo</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Commerce &amp; Restauration</t>
-        </is>
-      </c>
-      <c r="C35">
-        <v>7</v>
-      </c>
-      <c r="D35">
-        <v>7.9</v>
+          <t>Inactif / Retraité</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Feramanga Atsimo</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cultivateur exploitant</t>
-        </is>
-      </c>
-      <c r="C36">
-        <v>60</v>
-      </c>
-      <c r="D36">
-        <v>67.40000000000001</v>
+          <t>Ouvrier agricole</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Feramanga Atsimo</t>
+          <t>Avaradrano</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Elevage, Pêche &amp; Ress. nat.</t>
+          <t>Services &amp; Autres</t>
         </is>
       </c>
     </row>
@@ -960,14 +936,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
+          <t>Artisanat, BTP &amp; Transport</t>
         </is>
       </c>
       <c r="C38">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D38">
-        <v>11.2</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="39">
@@ -978,74 +954,74 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Services &amp; Autres</t>
-        </is>
+          <t>Commerce &amp; Restauration</t>
+        </is>
+      </c>
+      <c r="C39">
+        <v>7</v>
+      </c>
+      <c r="D39">
+        <v>7.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mangabe</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Artisanat, BTP &amp; Transport</t>
+          <t>Cultivateur exploitant</t>
         </is>
       </c>
       <c r="C40">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="D40">
-        <v>6.8</v>
+        <v>67.40000000000001</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mangabe</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Commerce &amp; Restauration</t>
+          <t>Elevage, Pêche &amp; Ress. nat.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Mangabe</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cultivateur exploitant</t>
+          <t>Ouvrier agricole</t>
         </is>
       </c>
       <c r="C42">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="D42">
-        <v>69.90000000000001</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mangabe</t>
+          <t>Feramanga Atsimo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Elevage, Pêche &amp; Ress. nat.</t>
-        </is>
-      </c>
-      <c r="C43">
-        <v>5</v>
-      </c>
-      <c r="D43">
-        <v>6.8</v>
+          <t>Services &amp; Autres</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1056,14 +1032,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
+          <t>Artisanat, BTP &amp; Transport</t>
         </is>
       </c>
       <c r="C44">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D44">
-        <v>11</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="45">
@@ -1074,98 +1050,86 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Services &amp; Autres</t>
+          <t>Commerce &amp; Restauration</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Artisanat, BTP &amp; Transport</t>
+          <t>Cultivateur exploitant</t>
         </is>
       </c>
       <c r="C46">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="D46">
-        <v>8.9</v>
+        <v>69.90000000000001</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Commerce &amp; Restauration</t>
+          <t>Elevage, Pêche &amp; Ress. nat.</t>
         </is>
       </c>
       <c r="C47">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="D47">
-        <v>5.5</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cultivateur exploitant</t>
-        </is>
-      </c>
-      <c r="C48">
-        <v>305</v>
-      </c>
-      <c r="D48">
-        <v>60.4</v>
+          <t>Inactif / Retraité</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Elevage, Pêche &amp; Ress. nat.</t>
+          <t>Ouvrier agricole</t>
         </is>
       </c>
       <c r="C49">
-        <v>31</v>
+        <v>8</v>
       </c>
       <c r="D49">
-        <v>6.1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tous</t>
+          <t>Mangabe</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Ouvrier agricole</t>
-        </is>
-      </c>
-      <c r="C50">
-        <v>63</v>
-      </c>
-      <c r="D50">
-        <v>12.5</v>
+          <t>Services &amp; Autres</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -1176,14 +1140,122 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
+          <t>Artisanat, BTP &amp; Transport</t>
+        </is>
+      </c>
+      <c r="C51">
+        <v>45</v>
+      </c>
+      <c r="D51">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Commerce &amp; Restauration</t>
+        </is>
+      </c>
+      <c r="C52">
+        <v>28</v>
+      </c>
+      <c r="D52">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Cultivateur exploitant</t>
+        </is>
+      </c>
+      <c r="C53">
+        <v>305</v>
+      </c>
+      <c r="D53">
+        <v>60.4</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Elevage, Pêche &amp; Ress. nat.</t>
+        </is>
+      </c>
+      <c r="C54">
+        <v>31</v>
+      </c>
+      <c r="D54">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Inactif / Retraité</t>
+        </is>
+      </c>
+      <c r="C55">
+        <v>16</v>
+      </c>
+      <c r="D55">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Ouvrier agricole</t>
+        </is>
+      </c>
+      <c r="C56">
+        <v>63</v>
+      </c>
+      <c r="D56">
+        <v>12.5</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Tous</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>Services &amp; Autres</t>
         </is>
       </c>
-      <c r="C51">
-        <v>33</v>
-      </c>
-      <c r="D51">
-        <v>6.5</v>
+      <c r="C57">
+        <v>17</v>
+      </c>
+      <c r="D57">
+        <v>3.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>